<commit_message>
Fill HSK1_parts_of_speech_5(201-250).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_5(201-250).xlsx
+++ b/HSK1_parts_of_speech_5(201-250).xlsx
@@ -601,6 +601,11 @@
           <t>текст учебника</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>текст (учебника)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +632,16 @@
           <t>рот</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>рот; уста</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>для предметов с ротовидной формой и отверстий: рот, ранец (一口锅); для глотков, кусков (吃一口)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +668,21 @@
           <t>кусок</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>кусок, глыба</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>для кусков и цельных предметов: кусок мыла, денег (一块钱), камень</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>как числительное «один» в разговорном языке: 一个→一块</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +709,21 @@
           <t>быстрый</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>свершать, резать (устар./книжн.)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>быстрый, скорый; шустрый</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>скорее, побыстрее (你快走吧)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +750,11 @@
           <t>приходить</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>приходить; прибывать</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +781,16 @@
           <t>прийти, прибыть</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>прибыть, прибыть куда-л.</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>словосочетание: глагол + направительное дополнение 到</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -757,6 +817,26 @@
           <t>старый</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>старик</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>стареть, взрослеть (他老了)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>старый, древний</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>часто префикс имён/прозвищ: 老王, 老师 — тогда не самостоятельная часть речи</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -783,6 +863,16 @@
           <t>пожилой человек</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>пожилой человек, старик</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>словосочетание: 老 (прил.) + 人 (сущ.)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -809,6 +899,16 @@
           <t>учитель</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>учитель, преподаватель</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>словосочетание (лексикализованное): 老 + 师</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -835,6 +935,16 @@
           <t>показатель завершённости действия (после сказуемого) или изменения ситуации (в конце предложения)</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>частица завершённости/изменения состояния (了)</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (служебная частица)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -861,6 +971,21 @@
           <t>усталый</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>уставать, утомляться</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>уставший, измученный</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>также читается léi — 累累 (нагромождённый), самостоятельно редко</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -887,6 +1012,16 @@
           <t>холодный</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>замораживать, мёрзнуть (冻冷/冷着了)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>холодный</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -913,6 +1048,21 @@
           <t>в</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>внутри, внутренность, нутро</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>внутри, в пределах чего-л.</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>лoкативное слово (方位词), требует опоры: 家里, 包里</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -939,6 +1089,21 @@
           <t>внутри</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>внутри, нутро</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>внутри</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>словосочетание/локаторная форма: 里 + 边</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -965,6 +1130,16 @@
           <t>два (количество)</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>оба, оба (两全其美 - редкое)</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>два (2 перед счётным словом: 两个人)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -996,6 +1171,21 @@
           <t>ноль</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>дробь, остаток (零头)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>небывалый, полный (零风险 - книжн.)</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>ноль, ноль (в числах, времени: 三点零五分)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1022,6 +1212,11 @@
           <t>шесть</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>шесть (6)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1048,6 +1243,16 @@
           <t>многоэтажное здание</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>здание, дом многоэтажный; этаж</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>для строений этажных: 一栋楼 (редко, чаще 栋)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1074,6 +1279,16 @@
           <t>верхний этаж</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>верхний этаж</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>словосочетание: 楼 + 上 (локатор)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1100,6 +1315,16 @@
           <t>нижний этаж</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>нижний этаж</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>словосочетание: 楼 + 下 (локатор)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1126,6 +1351,16 @@
           <t>дорога</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>путь, дорога, маршрут</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>для направлений пути: 一路顺风 (пожелание)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1152,6 +1387,16 @@
           <t>перекрёсток</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>перекрёсток, развилка, угол улицы</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>словосочетание: 路 + 口</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1178,6 +1423,16 @@
           <t>на дороге; в дороге</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>на дороге, в пути</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>словосочетание: 路 + 上</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1209,6 +1464,16 @@
           <t>мама</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>мама, матушка</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>повтор слога: 妈+妈 (детск./ласк.)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1235,6 +1500,16 @@
           <t>проезжая дорога, улица</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>шоссе, проезжая часть, улица</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>словосочетание: 马 + 路</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1261,6 +1536,21 @@
           <t>тотчас, скоро</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>седло и уздечка (устар.)</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>немедленно, тотчас, сейчас же</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>наречие из сочетания 马 (лошадь) + 上</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1287,6 +1577,16 @@
           <t>конечная частица вопросительных предложений</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>вопросительная частица (ли?, ли?) в конце вопроса без вопросительного слова</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (конечная частица)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1313,6 +1613,11 @@
           <t>покупать</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>покупать, приобретать</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1339,6 +1644,21 @@
           <t>медленный</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>замедлять, задерживать (慢待 - редкое)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>медленный, неторопливый</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>медленно, помедленнее (慢点走!)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1365,6 +1685,16 @@
           <t>занятой</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>суетиться, хлопотать (忙帮忙)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>занятой, загруженный</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1391,6 +1721,26 @@
           <t>шерсть; денежная единица в Китае (счётное слово)</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>шерсть, мех; волоски</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>истреблять, портить (毛笔 - кисть)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>волосатый, шершавый (毛的)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>для денег: мао (= 0.1 юаня)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1417,6 +1767,16 @@
           <t>не (отрицание)</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>тонуть, скрываться (淹没, 隐没)</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>не (перед 有 и глаголами: 我没有, 没去)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1443,6 +1803,16 @@
           <t>не иметь значения</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>не иметь значения, ничего страшного</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (вежливый ответ)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1469,6 +1839,16 @@
           <t>Ничего! Пустяки!</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>ничего особенного, пустяки</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (разг.)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1495,6 +1875,16 @@
           <t>ничего особенного</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>ничего, всё в порядке</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (разг., с эр-румянизмом)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1521,6 +1911,21 @@
           <t>не, не иметь</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>пустота, безденежье (穷没有 - редкое)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>не иметь, отсутствовать</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>не (завершённого действия: 没买)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1552,6 +1957,16 @@
           <t>младшая сестра</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>младшая сестра</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>словообразование: 妹 (сестра) + 子 суффикс</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1578,6 +1993,16 @@
           <t>дверь</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>дверь; вход, ворота</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>для дверей, приборов, навыков: 一门课 (курс), 一门手艺 (ремесло)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1604,6 +2029,16 @@
           <t>вход</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>у входа, преддверие, проход</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>словосочетание: 门 + 口; локативное значение «у входа»</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1630,6 +2065,16 @@
           <t>входной билет</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>входной билет, тариф</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>словосочетание: 门 (врата) + 票 (билет)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1661,6 +2106,16 @@
           <t>суффикс множественного числа (друзья)</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>суффикс множественного числа для лиц: 我们, 朋友们</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (суффикс, присоединяется к местоимениям и существительным-лицам)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1687,6 +2142,16 @@
           <t>варёный рис</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>варёный рис (зерновой), каша рисовая</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>словосочетание: 米 (рис) + 饭 (еда)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1713,6 +2178,16 @@
           <t>хлеб</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>хлеб (булка, батон)</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>словосочетание: 面 (мука) + 包 (выпечка)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1739,6 +2214,16 @@
           <t>лапша</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>лапша (длинные полоски теста)</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>словосочетание: 面 + 条儿 (полоска)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1765,6 +2250,16 @@
           <t>имя</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>имя, наименование</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>словосочетание: 名 (имя) + 字 (знак)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1791,6 +2286,21 @@
           <t>понимать; ясный</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>понимать, осознавать</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ясный, понятный (说明白)</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>также как комплемент результата: 听明白 (услышать и понять)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1817,6 +2327,16 @@
           <t>следующий год</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>следующий год</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>словосочетание: 明 (следующий) + 年</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1843,6 +2363,16 @@
           <t>завтра</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>завтрашний день</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>словосочетание: 明 + 天</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1869,6 +2399,21 @@
           <t>брать</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ручка, орудие (拿手 - мастерство)</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>брать, держать в руке; хватать</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>с помощью чего-л.; посредством (拿笔写字)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1893,6 +2438,11 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>который?</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>который? какой? (哪个, 哪儿); где? в вопросах (你在哪儿?)</t>
         </is>
       </c>
     </row>

</xml_diff>